<commit_message>
Actualizar datos e imagenes
</commit_message>
<xml_diff>
--- a/datos/productos.xlsx
+++ b/datos/productos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9af133bd758b7a26/Documentos/novacenter/datos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Documentos\novacenter\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{69EF108A-ED3E-45D6-ADFF-F02DA34B0CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E2F766-C778-424A-9EF5-E252725F88D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="0" windowWidth="21600" windowHeight="11385" xr2:uid="{24072905-EB78-43FF-AB26-A0FE06EC2951}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{24072905-EB78-43FF-AB26-A0FE06EC2951}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -20605,7 +20605,7 @@
         <v>1250</v>
       </c>
       <c r="L361">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="M361">
         <v>0</v>

</xml_diff>